<commit_message>
FK: Kampfmodul-Grenze bei Gute/Meisterliche-Formeln dokumentiert
- Klargestellt, dass die 18 fk_gute_*/fk_meisterlich_*-Formeln von der
  vollstaendigen Probe (Basis+Waffen-Modifikator+Entfernung) ausgehen -
  diese Zusammensetzung sowie die Probe<=0-Sonderregel (nur Meisterlich/
  Froehlich moeglich) gehoeren ins spaetere Kampfmodul, nicht in den
  Charakterbogen. Scope-Entscheidung, um Charaktererstellung zuerst
  fertigzustellen.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/werte 0.7-claude.xlsx
+++ b/werte 0.7-claude.xlsx
@@ -3965,6 +3965,11 @@
           <t>Fernkampf-Gute-Wert Blasrohre</t>
         </is>
       </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G95" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -3997,6 +4002,11 @@
           <t>Fernkampf-Gute-Wert Bögen</t>
         </is>
       </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G96" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4029,6 +4039,11 @@
           <t>Fernkampf-Gute-Wert Schusswaffen</t>
         </is>
       </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G97" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4061,6 +4076,11 @@
           <t>Fernkampf-Gute-Wert Wurfwaffen</t>
         </is>
       </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G98" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4093,6 +4113,11 @@
           <t>Fernkampf-Meisterliche-Wert Blasrohre</t>
         </is>
       </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G99" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4125,6 +4150,11 @@
           <t>Fernkampf-Meisterliche-Wert Bögen</t>
         </is>
       </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G100" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4157,6 +4187,11 @@
           <t>Fernkampf-Meisterliche-Wert Schusswaffen</t>
         </is>
       </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G101" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4189,6 +4224,11 @@
           <t>Fernkampf-Meisterliche-Wert Wurfwaffen</t>
         </is>
       </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G102" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4221,6 +4261,11 @@
           <t>Fernkampf-Spezialisierungs-Gute-Wert Armbrust</t>
         </is>
       </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G103" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4253,6 +4298,11 @@
           <t>Fernkampf-Spezialisierungs-Gute-Wert Blasrohre</t>
         </is>
       </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G104" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4285,6 +4335,11 @@
           <t>Fernkampf-Spezialisierungs-Gute-Wert Musketen</t>
         </is>
       </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G105" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4317,6 +4372,11 @@
           <t>Fernkampf-Spezialisierungs-Gute-Wert Pistolen</t>
         </is>
       </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G106" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4349,6 +4409,11 @@
           <t>Fernkampf-Spezialisierungs-Gute-Wert Bögen</t>
         </is>
       </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G107" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4381,6 +4446,11 @@
           <t>Fernkampf-Spezialisierungs-Meisterliche-Wert Armbrust</t>
         </is>
       </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G108" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4413,6 +4483,11 @@
           <t>Fernkampf-Spezialisierungs-Meisterliche-Wert Blasrohre</t>
         </is>
       </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G109" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4445,6 +4520,11 @@
           <t>Fernkampf-Spezialisierungs-Meisterliche-Wert Musketen</t>
         </is>
       </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G110" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4477,6 +4557,11 @@
           <t>Fernkampf-Spezialisierungs-Meisterliche-Wert Pistolen</t>
         </is>
       </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
+        </is>
+      </c>
       <c r="G111" t="inlineStr">
         <is>
           <t>Formel</t>
@@ -4507,6 +4592,11 @@
       <c r="C112" t="inlineStr">
         <is>
           <t>Fernkampf-Spezialisierungs-Meisterliche-Wert Bögen</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Diese Formel geht von der VOLLSTAENDIGEN Probe aus (Basiswert + Waffen-Modifikator + Entfernungs-Modifikator, siehe Waffentabellen z.B. NN_Feuerwaffen_1.1.xlsx). Die Berechnung dieser vollstaendigen Probe sowie die Sonderregel bei Probe&lt;=0 (nur Meisterlich=normaler Treffer bzw. Froehlich=guter Treffer moeglich) gehoeren ins zukuenftige Kampfmodul, nicht in den Charakterbogen - hier steht nur der Basismechanismus.</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">

</xml_diff>